<commit_message>
Modèle v6 : XGBoost sur l'enquête ménage, sans la grille Excel
- Le modèle apprend la décision de la vérification approfondie à partir des
  72 réponses de l'enquête ménage. La grille Excel, son score et son seuil ne
  sont plus donnés au modèle (ils servent seulement de comparaison).
- Nouvelles données simulées (notebooks/generateur_ciblage_v6.py) et notebook
  ciblage_avec_ml_v6.ipynb : 7 modèles comparés, validation croisée, SHAP,
  comparaison avec la grille. XGBoost en test : accuracy 98,1 %, F1 96,9 %,
  rappel 96,2 %, précision 97,6 % ; jamais sous 96,4 % en validation croisée.
- Formulaire Kobo régénéré : 73 questions en 10 groupes, contrôles de cohérence.
- API et dashboard : explication par réponse et par thème, zone grise selon la
  probabilité, sélection sous budget classée par l'indice du modèle.
- LightGBM remplacé par XGBoost ; tests et README mis à jour.
</commit_message>
<xml_diff>
--- a/kobo/formulaire_ciblage_menages.xlsx
+++ b/kobo/formulaire_ciblage_menages.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,17 +424,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
     <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="39" customWidth="1" min="8" max="8"/>
+    <col width="63" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -837,7 +837,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Profil du ménage</t>
+          <t>Profil</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -955,17 +955,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>select_one sexe_chef_menage</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sexe_chef_menage</t>
+          <t>nombre_deplacements_12m</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sexe du chef de ménage</t>
+          <t>Combien de fois le ménage a-t-il dû fuir au cours des 12 derniers mois ?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -974,25 +974,37 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 15</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 15</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>${statut_menage} = 'deplace' or ${statut_menage} = 'retourne'</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one sexe_chef_menage</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>age_chef_menage</t>
+          <t>sexe_chef_menage</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Âge du chef de ménage (années)</t>
+          <t>Sexe du chef de ménage</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1001,16 +1013,8 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>. &gt;= 10 and . &lt;= 110</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>La valeur doit être comprise entre 10 et 110</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
     </row>
@@ -1022,19 +1026,15 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>taille_menage</t>
+          <t>age_chef_menage</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nombre de personnes dans le ménage</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Toutes les personnes qui vivent et mangent ensemble, chef de ménage compris</t>
-        </is>
-      </c>
+          <t>Âge du chef de ménage (années)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1042,12 +1042,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>. &gt;= 1 and . &lt;= 40</t>
+          <t>. &gt;= 10 and . &lt;= 110</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>La valeur doit être comprise entre 1 et 40</t>
+          <t>La valeur doit être comprise entre 10 et 110</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1056,17 +1056,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one etat_civil_chef</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>enfants_moins_5</t>
+          <t>etat_civil_chef</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nombre d'enfants de moins de 5 ans dans le ménage</t>
+          <t>État civil du chef de ménage</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1075,29 +1075,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 20 and . &lt; ${taille_menage}</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>La valeur doit être comprise entre 0 et 20. Doit être inférieur à la taille du ménage (le chef de ménage en fait partie)</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
+          <t>select_one instruction_chef</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>instruction_chef</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Niveau d'instruction du chef de ménage</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -1106,98 +1110,98 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>vulnerabilites</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Vulnérabilités</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>${consentement} = 'oui'</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>membre_handicap</t>
+          <t>composition</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Un membre du ménage vit-il avec un handicap ?</t>
+          <t>Composition</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>membre_maladie_chronique</t>
+          <t>taille_menage</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Un membre du ménage a-t-il une maladie chronique ?</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>Nombre de personnes dans le ménage</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Toutes les personnes qui vivent et mangent ensemble, chef de ménage compris</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 40</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 1 et 40</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>femme_enceinte_allaitante</t>
+          <t>enfants_moins_5</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Le ménage a-t-il une femme enceinte ou allaitante ?</t>
+          <t>Nombre d'enfants de moins de 5 ans</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1206,25 +1210,33 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 20</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 20</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>select_one oui_non</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>enfant_non_accompagne_heberge</t>
+          <t>enfants_5_17</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Le ménage héberge-t-il un enfant non accompagné ou séparé ?</t>
+          <t>Nombre d'enfants de 5 à 17 ans</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1233,67 +1245,103 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 25</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 25</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>personnes_60_plus</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Nombre de personnes de 60 ans ou plus</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 10 and . + ${enfants_moins_5} + ${enfants_5_17} &lt;= ${taille_menage}</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 10. Enfants et personnes âgées dépassent la taille du ménage</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>logement</t>
+          <t>enfants_non_scolarises</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Logement et biens</t>
+          <t>Parmi les enfants de 5 à 17 ans, combien ne vont pas à l'école ?</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>${consentement} = 'oui'</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 25 and . &lt;= ${enfants_5_17}</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 25. Ne peut pas dépasser le nombre d'enfants de 5 à 17 ans</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>select_one type_logement</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>type_logement</t>
+          <t>femme_enceinte_allaitante</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Type de logement actuel</t>
+          <t>Le ménage a-t-il une femme enceinte ou allaitante ?</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1310,39 +1358,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>articles_essentiels</t>
+          <t>membre_handicap</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Combien de ces 5 articles le ménage possède-t-il en quantité suffisante ?</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Couvertures, nattes, bidons, ustensiles de cuisine, moustiquaires</t>
-        </is>
-      </c>
+          <t>Un membre du ménage vit-il avec un handicap ?</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 5</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>La valeur doit être comprise entre 0 et 5</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
     </row>
@@ -1354,12 +1390,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>possede_betail</t>
+          <t>membre_maladie_chronique</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Le ménage possède-t-il du bétail (au moins 2 chèvres ou équivalent) ?</t>
+          <t>Un membre du ménage a-t-il une maladie chronique ?</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1376,13 +1412,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>enfant_non_accompagne_heberge</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Le ménage héberge-t-il un enfant non accompagné ou séparé ?</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
@@ -1391,71 +1439,59 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>begin_group</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>alimentation_revenus</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Alimentation et revenus</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>${consentement} = 'oui'</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>select_one repas_par_jour</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>repas_par_jour</t>
+          <t>logement</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Nombre de repas pris par jour par les adultes (7 derniers jours)</t>
+          <t>Logement et biens</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one type_logement</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>jours_sans_nourriture_7j</t>
+          <t>type_logement</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Au cours des 7 derniers jours, combien de jours le ménage n'a-t-il rien eu à manger ?</t>
+          <t>Type de logement actuel</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1464,33 +1500,25 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 7</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>La valeur doit être comprise entre 0 et 7</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>select_one source_revenu</t>
+          <t>select_one statut_occupation</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>source_revenu</t>
+          <t>statut_occupation</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Principale source de revenu du ménage</t>
+          <t>Statut d'occupation du logement</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1507,43 +1535,79 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>nombre_pieces</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Nombre de pièces pour dormir</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0 si le ménage dort à la belle étoile</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 15</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 15</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>assistance</t>
+          <t>articles_essentiels</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Assistance reçue</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>${consentement} = 'oui'</t>
-        </is>
-      </c>
+          <t>Combien de ces 5 articles le ménage possède-t-il en quantité suffisante ?</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Couvertures, nattes, bidons, ustensiles de cuisine, moustiquaires</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 5</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 5</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
@@ -1554,12 +1618,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>assistance_3_derniers_mois</t>
+          <t>possede_betail</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Le ménage a-t-il reçu une assistance humanitaire au cours des 3 derniers mois ?</t>
+          <t>Le ménage possède-t-il du bétail (au moins 2 chèvres ou équivalent) ?</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1576,17 +1640,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>select_one type_assistance_recue</t>
+          <t>select_one oui_non</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>type_assistance_recue</t>
+          <t>acces_terre_cultivable</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Quel type d'assistance ?</t>
+          <t>Le ménage a-t-il accès à une terre qu'il peut cultiver cette saison ?</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1597,23 +1661,31 @@
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>${assistance_3_derniers_mois} = 'oui'</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>toit_etanche</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Le toit du logement protège-t-il de la pluie ?</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
@@ -1622,29 +1694,1897 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one source_eclairage</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>fin</t>
+          <t>source_eclairage</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Merci. L'éligibilité sera calculée à la réception de la soumission et revue par l'équipe de ciblage.</t>
+          <t>Principale source d'éclairage du ménage</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>possede_telephone</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Un membre du ménage possède-t-il un téléphone ?</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>eau_hygiene</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Eau et hygiène</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
         <is>
           <t>${consentement} = 'oui'</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>select_one source_eau</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>source_eau</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Principale source d'eau de boisson</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>temps_collecte_eau_min</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Temps nécessaire pour aller chercher l'eau et revenir (minutes)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 600</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 600</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>select_one type_latrine</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>type_latrine</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Type de latrine utilisée</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>savon_disponible</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Y a-t-il du savon dans le ménage aujourd'hui ?</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>sante</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Santé et nutrition</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>enfant_malade_2_semaines</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Un enfant de moins de 5 ans a-t-il eu la diarrhée ou de la fièvre ces 2 dernières semaines ?</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>« Non » si le ménage n'a pas d'enfant de moins de 5 ans</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>select_one acces_soins</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>acces_soins</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>La dernière fois qu'un membre a eu besoin de soins, a-t-il pu les obtenir ?</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>select_one vaccination_enfants_a_jour</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>vaccination_enfants_a_jour</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Les enfants de moins de 5 ans ont-ils tous leur carte de vaccination à jour ?</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>enfant_malnutrition_depiste</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Un enfant du ménage a-t-il été dépisté malnutri (périmètre brachial jaune ou rouge) ?</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>alimentation</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Alimentation</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>jours_cereales</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : céréales, tubercules (maïs, manioc, riz, banane plantain) ?</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>jours_legumineuses</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : légumineuses (haricots, petits pois, arachides) ?</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>jours_lait</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : lait ou produits laitiers ?</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>jours_viande_poisson</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : viande, poisson ou œufs ?</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>jours_legumes</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : légumes ou feuilles (sombé, amarante) ?</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>jours_fruits</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : fruits ?</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>jours_huile</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : huile ou graisse ?</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>jours_sucre</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il mangé : sucre ou miel ?</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>stock_nourriture_jours</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Pour combien de jours le ménage a-t-il des réserves de nourriture ?</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>0 si aucune réserve</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 365</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 365</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>select_one repas_par_jour</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>repas_par_jour</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Nombre de repas pris par jour par les adultes (7 derniers jours)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>jours_sans_nourriture_7j</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage n'a-t-il rien eu à manger ?</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>adaptation</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Stratégies d'adaptation</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>rcsi_aliments_moins_chers</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il dû consommer des aliments moins préférés ou moins chers ?</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>rcsi_emprunt_nourriture</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il dû emprunter de la nourriture ou compter sur l'aide de proches ?</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>rcsi_reduction_portions</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il dû réduire la taille des portions ?</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>rcsi_adultes_pour_enfants</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il dû réduire la consommation des adultes pour nourrir les enfants ?</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>rcsi_moins_de_repas</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Au cours des 7 derniers jours, combien de jours le ménage a-t-il dû réduire le nombre de repas ?</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>0 à 7 jours</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 7</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 7</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>lcs_emprunt_argent</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû emprunter de l'argent ou acheter à crédit faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>lcs_vente_biens_menagers</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû vendre des biens du ménage (meubles, radio, ustensiles) faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>lcs_consommation_semences</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû consommer les semences prévues pour la prochaine saison faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>lcs_reduction_depenses_sante</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû réduire les dépenses de santé ou d'éducation faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>lcs_retrait_enfants_ecole</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû retirer des enfants de l'école faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>lcs_vente_derniere_femelle</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû vendre la dernière femelle reproductrice (chèvre, vache) faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>lcs_vente_maison_terre</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû vendre la maison ou la terre faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>lcs_mendicite</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû mendier faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>lcs_travail_enfants</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Au cours des 30 derniers jours, le ménage a-t-il dû envoyer des enfants travailler faute de nourriture ou d'argent ?</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>moyens_existence</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Moyens d'existence</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>select_one source_revenu</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>source_revenu</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Principale source de revenu du ménage</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>membres_avec_revenu</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Combien de membres du ménage ont gagné de l'argent au cours des 30 derniers jours ?</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 20</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 20</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>perte_revenu_6_mois</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Le ménage a-t-il perdu sa principale source de revenu au cours des 6 derniers mois ?</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>revenu_30j_usd</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Revenu total du ménage au cours des 30 derniers jours (en dollars US)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Convertir les francs congolais en dollars</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 5000</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 5000</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>part_depenses_alimentation_pct</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Part des dépenses du ménage consacrée à la nourriture (%)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 100</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 100</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>dette_usd</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Montant des dettes actuelles du ménage (en dollars US)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>0 si aucune dette</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 20000</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>La valeur doit être comprise entre 0 et 20000</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>epargne_disponible</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Le ménage a-t-il de l'épargne (argent mis de côté, tontine, mobile money) ?</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>protection</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>incident_securite_3_mois</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Un membre du ménage a-t-il subi un incident de sécurité ces 3 derniers mois ?</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Vol, agression, extorsion, enlèvement, violence</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>biens_perdus_crise</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Le ménage a-t-il perdu des biens à cause de la crise (pillage, incendie, destruction) ?</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>membre_disparu_detenu</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Un membre du ménage a-t-il disparu, été enlevé ou détenu depuis le début de la crise ?</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>documents_identite</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Le chef de ménage possède-t-il une pièce d'identité ou un document d'électeur ?</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>restriction_mouvements</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Les membres du ménage évitent-ils certains lieux (champs, marché) par peur pour leur sécurité ?</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr"/>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>begin_group</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>assistance</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Assistance</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>select_one oui_non</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>assistance_3_derniers_mois</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Le ménage a-t-il reçu une assistance humanitaire au cours des 3 derniers mois ?</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>select_one type_assistance_recue</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>type_assistance_recue</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Quel type d'assistance ?</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>${assistance_3_derniers_mois} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>fin</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Merci. L'éligibilité sera calculée à la réception de la soumission et revue par l'équipe de ciblage.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>${consentement} = 'oui'</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1657,12 +3597,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1923,304 +3863,831 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>type_logement</t>
+          <t>etat_civil_chef</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison_correcte</t>
+          <t>marie</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Maison en bon état</t>
+          <t>Marié(e) / union libre</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>type_logement</t>
+          <t>etat_civil_chef</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>maison_endommagee</t>
+          <t>celibataire</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Maison endommagée</t>
+          <t>Célibataire</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>type_logement</t>
+          <t>etat_civil_chef</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>heberge_famille</t>
+          <t>veuf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hébergé par une famille</t>
+          <t>Veuf / veuve</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>type_logement</t>
+          <t>etat_civil_chef</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>abri_fortune</t>
+          <t>divorce_separe</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Abri de fortune</t>
+          <t>Divorcé(e) / séparé(e)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>type_logement</t>
+          <t>instruction_chef</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sans_abri</t>
+          <t>aucun</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sans abri</t>
+          <t>Aucun</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>repas_par_jour</t>
+          <t>instruction_chef</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>primaire</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1 repas ou moins</t>
+          <t>Primaire</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>repas_par_jour</t>
+          <t>instruction_chef</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>secondaire</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2 repas</t>
+          <t>Secondaire</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>repas_par_jour</t>
+          <t>instruction_chef</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>superieur</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3 repas ou plus</t>
+          <t>Supérieur</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>source_revenu</t>
+          <t>type_logement</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>salaire_regulier</t>
+          <t>maison_correcte</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Salaire régulier</t>
+          <t>Maison en bon état</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>source_revenu</t>
+          <t>type_logement</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>petit_commerce</t>
+          <t>maison_endommagee</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Petit commerce</t>
+          <t>Maison endommagée</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>source_revenu</t>
+          <t>type_logement</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>heberge_famille</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Hébergé par une famille</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>source_revenu</t>
+          <t>type_logement</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>travail_journalier</t>
+          <t>abri_fortune</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Travail journalier</t>
+          <t>Abri de fortune</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>source_revenu</t>
+          <t>type_logement</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>aucun_revenu</t>
+          <t>sans_abri</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Aucun revenu / mendicité</t>
+          <t>Sans abri</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>type_assistance_recue</t>
+          <t>statut_occupation</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>vivres</t>
+          <t>proprietaire</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Vivres</t>
+          <t>Propriétaire</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>type_assistance_recue</t>
+          <t>statut_occupation</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>cash</t>
+          <t>locataire</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Locataire</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>type_assistance_recue</t>
+          <t>statut_occupation</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>articles_menagers</t>
+          <t>heberge_gratuit</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Articles ménagers</t>
+          <t>Hébergé gratuitement</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>type_assistance_recue</t>
+          <t>statut_occupation</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>abri</t>
+          <t>site_deplaces</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Abri</t>
+          <t>Site ou centre collectif de déplacés</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>source_eclairage</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>electricite</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Électricité (réseau)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>source_eclairage</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>solaire</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Panneau ou lampe solaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>source_eclairage</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>lampe_torche</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lampe torche, bougie, lampe à pétrole</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>source_eclairage</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>aucune</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>source_eau</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>robinet</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Robinet / borne fontaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>source_eau</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>puits_protege</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Puits ou source aménagés</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>source_eau</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>source_non_protegee</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Puits ou source non protégés</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>source_eau</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>eau_surface</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Eau de surface (rivière, lac)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>type_latrine</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>privee</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Latrine du ménage</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>type_latrine</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>partagee</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Latrine partagée</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>type_latrine</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>aucune</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Aucune (défécation à l'air libre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>acces_soins</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>acces_soins</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>non_cout</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Non, trop cher</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>acces_soins</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>non_distance</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Non, trop loin</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>acces_soins</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>non_insecurite</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Non, à cause de l'insécurité</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>acces_soins</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>pas_besoin</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Pas de besoin de soins</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>vaccination_enfants_a_jour</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>vaccination_enfants_a_jour</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>vaccination_enfants_a_jour</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>pas_enfant</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Pas d'enfant de moins de 5 ans</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>repas_par_jour</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1 repas ou moins</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>repas_par_jour</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2 repas</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>repas_par_jour</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>3 repas ou plus</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>source_revenu</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>salaire_regulier</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Salaire régulier</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>source_revenu</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>petit_commerce</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Petit commerce</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>source_revenu</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>agriculture</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>source_revenu</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>travail_journalier</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Travail journalier</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>source_revenu</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>aucun_revenu</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Aucun revenu / mendicité</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>type_assistance_recue</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>vivres</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Vivres</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>type_assistance_recue</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>type_assistance_recue</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>articles_menagers</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Articles ménagers</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>type_assistance_recue</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>abri</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Abri</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>type_assistance_recue</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>autre</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>Autre</t>
         </is>
@@ -2281,7 +4748,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026102219</t>
+          <t>2026102400</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>